<commit_message>
Report net profit (after expenses) in dashboard shop profits export
</commit_message>
<xml_diff>
--- a/price list.xlsx
+++ b/price list.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="141">
   <si>
     <t>Product</t>
   </si>
@@ -391,19 +391,25 @@
     <t>mInutemaid Small</t>
   </si>
   <si>
+    <t>45</t>
+  </si>
+  <si>
     <t>mInutemaid Big</t>
   </si>
   <si>
+    <t>100</t>
+  </si>
+  <si>
     <t>Dasani Small</t>
   </si>
   <si>
-    <t>40</t>
+    <t>33</t>
+  </si>
+  <si>
+    <t>50</t>
   </si>
   <si>
     <t>Dasani Big</t>
-  </si>
-  <si>
-    <t>50</t>
   </si>
   <si>
     <t>Lemonade</t>
@@ -1132,8 +1138,8 @@
       <c r="A21" t="s">
         <v>29</v>
       </c>
-      <c r="B21">
-        <v>100</v>
+      <c r="B21" t="s">
+        <v>7</v>
       </c>
       <c r="C21">
         <v>160</v>
@@ -2226,6 +2232,9 @@
       <c r="A109" t="s">
         <v>124</v>
       </c>
+      <c r="B109" t="s">
+        <v>125</v>
+      </c>
       <c r="C109">
         <v>80</v>
       </c>
@@ -2235,7 +2244,10 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>125</v>
+        <v>126</v>
+      </c>
+      <c r="B110" t="s">
+        <v>127</v>
       </c>
       <c r="C110">
         <v>160</v>
@@ -2246,13 +2258,13 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B111" t="s">
-        <v>127</v>
-      </c>
-      <c r="C111">
-        <v>70</v>
+        <v>129</v>
+      </c>
+      <c r="C111" t="s">
+        <v>130</v>
       </c>
       <c r="D111" t="s">
         <v>110</v>
@@ -2260,10 +2272,10 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B112" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C112">
         <v>100</v>
@@ -2274,13 +2286,13 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B113" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C113" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D113" t="s">
         <v>110</v>
@@ -2288,10 +2300,10 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B114" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C114">
         <v>70</v>
@@ -2302,7 +2314,7 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C115">
         <v>100</v>
@@ -2313,10 +2325,10 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B116" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C116">
         <v>30</v>
@@ -2327,7 +2339,7 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B117" t="s">
         <v>120</v>

</xml_diff>

<commit_message>
Remove Guinness, Torrero and Afia from the master price list
The three products were only in the master sheet and never given shop
sheets, so remove them everywhere the sync reads until they are ready
to be sold properly.

🤖 Generated with Codebuff 🤖

Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/price list.xlsx
+++ b/price list.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D121"/>
+  <dimension ref="A1:D118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="2"/>
@@ -999,14 +999,14 @@
     <row r="28" ht="18.75" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Afia</t>
+          <t>Chrome brandy</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>60</v>
+        <v>225</v>
       </c>
       <c r="C28" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1015,59 +1015,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Chrome brandy</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>225</v>
-      </c>
-      <c r="C29" t="n">
-        <v>300</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>250ml</t>
-        </is>
-      </c>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Brand 350ml</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Torrero</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>280</v>
-      </c>
-      <c r="C30" t="n">
-        <v>400</v>
+          <t xml:space="preserve">Jameson </t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>250ml</t>
+          <t>350ml</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Brand 350ml</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="n"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Richot</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>800</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>350ml</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jameson </t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
+          <t>Black&amp;white</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1100</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1078,11 +1072,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Richot</t>
-        </is>
+          <t>Gilbeys</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>580</v>
       </c>
       <c r="C33" t="n">
-        <v>800</v>
+        <v>850</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1093,11 +1090,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Black&amp;white</t>
+          <t>Smirnoff</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1100</v>
+        <v>850</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1108,14 +1105,16 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Gilbeys</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>580</v>
+          <t>Kibao</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
       </c>
       <c r="C35" t="n">
-        <v>850</v>
+        <v>500</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1126,11 +1125,18 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Smirnoff</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>850</v>
+          <t>Hunters</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>412</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>650</t>
+        </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1141,71 +1147,55 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Kibao</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
+          <t>Viceroy</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>575</v>
       </c>
       <c r="C37" t="n">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>350ml</t>
+          <t>375ml</t>
         </is>
       </c>
     </row>
     <row r="38" ht="22.5" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Hunters</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>412</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>650</t>
-        </is>
+          <t>VAT 69</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>800</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>350ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Viceroy</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>575</v>
-      </c>
-      <c r="C39" t="n">
-        <v>800</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>375ml</t>
-        </is>
-      </c>
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Brand 750ml</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>VAT 69</t>
-        </is>
+          <t>Kc smooth</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>703</v>
       </c>
       <c r="C40" t="n">
-        <v>800</v>
+        <v>1000</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1214,24 +1204,36 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>Brand 750ml</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="n"/>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>KC. Pineapple</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>703</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>750ml</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kc smooth</t>
+          <t>Kc.Ginger</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>703</v>
       </c>
-      <c r="C42" t="n">
-        <v>1000</v>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1242,14 +1244,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>KC. Pineapple</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>703</v>
+          <t>V&amp;A</t>
+        </is>
       </c>
       <c r="C43" t="n">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1260,15 +1259,15 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kc.Ginger</t>
+          <t>Hunters</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>703</v>
+        <v>900</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1300</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1280,11 +1279,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>V&amp;A</t>
+          <t xml:space="preserve">All seasons </t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>900</v>
+        <v>1200</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1295,16 +1294,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Hunters</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>900</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
+          <t>Kenya king</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1000</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1315,11 +1309,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">All seasons </t>
+          <t>Chrome Vodka</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>610</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1330,7 +1329,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kenya king</t>
+          <t>Chrome Gin</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>610</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1345,16 +1349,11 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Chrome Vodka</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>610</t>
+          <t>Imperial Blue</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1365,16 +1364,11 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Chrome Gin</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>610</t>
+          <t>Origin</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1385,11 +1379,11 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Imperial Blue</t>
+          <t>4th street</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1600</v>
+        <v>1100</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1400,11 +1394,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Origin</t>
+          <t>jameson 1l</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1100</v>
+        <v>3000</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1415,11 +1409,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>4th street</t>
+          <t>Jameson 750ml</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1100</v>
+        <v>2500</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -1430,11 +1424,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>jameson 1l</t>
+          <t>William Lawsons</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -1445,11 +1439,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Jameson 750ml</t>
+          <t>viceroy</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1200</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1460,11 +1459,14 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>William Lawsons</t>
-        </is>
+          <t>Black&amp;white</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1000</v>
       </c>
       <c r="C56" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1475,13 +1477,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>viceroy</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
+          <t>Gilbeys</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>580</v>
       </c>
       <c r="C57" t="n">
         <v>1500</v>
@@ -1495,14 +1495,14 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Black&amp;white</t>
+          <t>Captain Morgan</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1000</v>
+        <v>910</v>
       </c>
       <c r="C58" t="n">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1513,14 +1513,14 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Gilbeys</t>
+          <t>County</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>580</v>
+        <v>670</v>
       </c>
       <c r="C59" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1531,14 +1531,11 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Captain Morgan</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>910</v>
+          <t>Smirnoff</t>
+        </is>
       </c>
       <c r="C60" t="n">
-        <v>1200</v>
+        <v>1400</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1549,11 +1546,8 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>670</v>
+          <t>Kibao</t>
+        </is>
       </c>
       <c r="C61" t="n">
         <v>1000</v>
@@ -1567,11 +1561,18 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Smirnoff</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>1400</v>
+          <t>General Meakings</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -1582,11 +1583,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Kibao</t>
+          <t>Amarula 1ltr</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -1597,18 +1598,11 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>General Meakings</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>900</t>
-        </is>
+          <t>Amarula 750</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>2500</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1619,11 +1613,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Amarula 1ltr</t>
+          <t>Best Gin</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3000</v>
+        <v>950</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -1634,11 +1628,11 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Amarula 750</t>
+          <t>Best Whisky</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2500</v>
+        <v>1200</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -1649,11 +1643,11 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Best Gin</t>
+          <t>Red label 750</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>950</v>
+        <v>2200</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -1664,11 +1658,11 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Best Whisky</t>
+          <t>Red label 375ml</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1200</v>
+        <v>1300</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -1679,11 +1673,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Red label 750</t>
+          <t>Red Label 1 ltr</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2200</v>
+        <v>2600</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -1694,11 +1688,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Red label 375ml</t>
+          <t>Black Label 375ml</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1300</v>
+        <v>2250</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -1709,11 +1703,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Red Label 1 ltr</t>
+          <t>Black Label 750ml</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2600</v>
+        <v>3500</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -1724,11 +1718,11 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Black Label 375ml</t>
+          <t>Black Label 1ltr</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2250</v>
+        <v>4000</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -1739,11 +1733,11 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Black Label 750ml</t>
+          <t>Drostody hol</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>3500</v>
+        <v>1000</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -1754,11 +1748,11 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Black Label 1ltr</t>
+          <t>Richot</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>4000</v>
+        <v>1500</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -1769,11 +1763,11 @@
     <row r="75" ht="22.5" customHeight="1">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Drostody hol</t>
+          <t>VAT 69</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1000</v>
+        <v>1800</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -1782,54 +1776,60 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Richot</t>
-        </is>
-      </c>
-      <c r="C76" t="n">
-        <v>1500</v>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>750ml</t>
-        </is>
-      </c>
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>Cans</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>VAT 69</t>
-        </is>
+          <t xml:space="preserve">Guarana </t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>175</v>
       </c>
       <c r="C77" t="n">
-        <v>1800</v>
+        <v>250</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>cans</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="5" t="inlineStr">
-        <is>
-          <t>Cans</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="n"/>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Guarana Black</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>175</v>
+      </c>
+      <c r="C78" t="n">
+        <v>250</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>cans</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guarana </t>
+          <t>Guiness</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>175</v>
+        <v>215</v>
       </c>
       <c r="C79" t="n">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -1840,14 +1840,14 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Guarana Black</t>
+          <t>Tusker</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>175</v>
+        <v>198</v>
       </c>
       <c r="C80" t="n">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -1858,11 +1858,11 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Guiness</t>
+          <t>Tusker Malt</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C81" t="n">
         <v>300</v>
@@ -1876,11 +1876,11 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Guinness</t>
+          <t>Tusker Lite</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="C82" t="n">
         <v>300</v>
@@ -1894,11 +1894,11 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Tusker</t>
+          <t xml:space="preserve">Tusker cider </t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>198</v>
+        <v>232</v>
       </c>
       <c r="C83" t="n">
         <v>300</v>
@@ -1912,11 +1912,8 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Tusker Malt</t>
-        </is>
-      </c>
-      <c r="B84" t="n">
-        <v>200</v>
+          <t>Snapp</t>
+        </is>
       </c>
       <c r="C84" t="n">
         <v>300</v>
@@ -1930,11 +1927,11 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Tusker Lite</t>
+          <t>pineapple Punch</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="C85" t="n">
         <v>300</v>
@@ -1948,11 +1945,8 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tusker cider </t>
-        </is>
-      </c>
-      <c r="B86" t="n">
-        <v>232</v>
+          <t>Faxe</t>
+        </is>
       </c>
       <c r="C86" t="n">
         <v>300</v>
@@ -1966,11 +1960,11 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Snapp</t>
+          <t>Redbull</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -1981,14 +1975,11 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>pineapple Punch</t>
-        </is>
-      </c>
-      <c r="B88" t="n">
-        <v>175</v>
+          <t xml:space="preserve">Delmonte </t>
+        </is>
       </c>
       <c r="C88" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -1999,7 +1990,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Faxe</t>
+          <t>Balozi</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>245</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -2014,11 +2010,18 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Redbull</t>
-        </is>
-      </c>
-      <c r="C90" t="n">
-        <v>250</v>
+          <t>Balozi Bottle</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>169</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -2029,11 +2032,14 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delmonte </t>
-        </is>
+          <t>Whitecup</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>215</v>
       </c>
       <c r="C91" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -2044,16 +2050,14 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Balozi</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>245</t>
-        </is>
+          <t>Caprice</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>600</v>
       </c>
       <c r="C92" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2064,18 +2068,14 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Balozi Bottle</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>169</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
+          <t>Pilsner Bottle</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>200</v>
+      </c>
+      <c r="C93" t="n">
+        <v>270</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -2086,14 +2086,18 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Whitecup</t>
-        </is>
-      </c>
-      <c r="B94" t="n">
-        <v>215</v>
-      </c>
-      <c r="C94" t="n">
-        <v>300</v>
+          <t>Heineken</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>169</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2104,29 +2108,31 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Caprice</t>
+          <t>Tusker Bottle</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>600</v>
+        <v>198</v>
       </c>
       <c r="C95" t="n">
-        <v>800</v>
+        <v>270</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>cans</t>
+          <t>Bottle</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Pilsner Bottle</t>
-        </is>
-      </c>
-      <c r="B96" t="n">
-        <v>200</v>
+          <t>Guiness</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
       </c>
       <c r="C96" t="n">
         <v>270</v>
@@ -2140,17 +2146,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Heineken</t>
+          <t>Guiness Bottle</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>204</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>270</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2162,30 +2168,30 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Tusker Bottle</t>
+          <t xml:space="preserve">Tusker cider </t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>198</v>
+        <v>234</v>
       </c>
       <c r="C98" t="n">
         <v>270</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Bottle</t>
+          <t>cans</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Guiness</t>
+          <t xml:space="preserve">Pilsner </t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>195</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -2200,83 +2206,80 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Guiness Bottle</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>204</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>270</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>cans</t>
+          <t>pilsner bottle</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tusker cider </t>
-        </is>
-      </c>
-      <c r="B101" t="n">
-        <v>234</v>
+          <t>White Cup Bottle</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
       </c>
       <c r="C101" t="n">
         <v>270</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>cans</t>
+          <t>soda</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilsner </t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>195</t>
+          <t xml:space="preserve">Kingfisher </t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>270</v>
+        <v>300</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>cans</t>
+          <t>soda</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>pilsner bottle</t>
+          <t>Soda 500ml</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>soda</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>White Cup Bottle</t>
+          <t>Soda 350ml</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>41</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>270</v>
+        <v>50</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -2287,11 +2290,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kingfisher </t>
+          <t>Soda 300ml</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>32</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -2302,18 +2310,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Soda 500ml</t>
+          <t>Soda 200ml</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>30</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -2324,16 +2330,11 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Soda 350ml</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>41</t>
+          <t>Soda 1.25ltrs</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -2344,16 +2345,11 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Soda 300ml</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>32</t>
+          <t>soda 1ltr</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>40</v>
+        <v>150</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -2364,16 +2360,11 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Soda 200ml</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>25</t>
+          <t>Soda 2ltrs</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>30</v>
+        <v>200</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -2384,11 +2375,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Soda 1.25ltrs</t>
+          <t>mInutemaid Small</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>45</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>180</v>
+        <v>80</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -2399,11 +2395,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>soda 1ltr</t>
+          <t>mInutemaid Big</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>100</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -2414,11 +2415,18 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Soda 2ltrs</t>
-        </is>
-      </c>
-      <c r="C112" t="n">
-        <v>200</v>
+          <t>Dasani Small</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -2429,16 +2437,16 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>mInutemaid Small</t>
+          <t>Dasani Big</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -2449,16 +2457,18 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>mInutemaid Big</t>
+          <t>Lemonade</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="C114" t="n">
-        <v>160</v>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -2469,18 +2479,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Dasani Small</t>
+          <t>predator</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>70</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -2491,12 +2499,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Dasani Big</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>50</t>
+          <t>Kiss</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -2511,18 +2514,16 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Lemonade</t>
+          <t>Glacier Small</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>30</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -2533,73 +2534,18 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>predator</t>
+          <t>Glacier Big</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="D118" t="inlineStr">
-        <is>
-          <t>soda</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>Kiss</t>
-        </is>
-      </c>
-      <c r="C119" t="n">
-        <v>100</v>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>soda</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>Glacier Small</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C120" t="n">
-        <v>30</v>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>soda</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>Glacier Big</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="C121" t="n">
-        <v>50</v>
-      </c>
-      <c r="D121" t="inlineStr">
         <is>
           <t>soda</t>
         </is>

</xml_diff>